<commit_message>
Update reports 8th Oct morning
</commit_message>
<xml_diff>
--- a/data/Oct/InternalDailyReport_Oct.xlsx
+++ b/data/Oct/InternalDailyReport_Oct.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Oct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE64E91-6610-407C-B341-2F5663DF8B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C046F6-7BC3-4544-A595-BD982D1D058E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="23" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="03-10" sheetId="26" r:id="rId4"/>
     <sheet name="05-10" sheetId="27" r:id="rId5"/>
     <sheet name="06-10" sheetId="28" r:id="rId6"/>
+    <sheet name="07-10" sheetId="29" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01-10'!$A$2:$P$53</definedName>
@@ -26,6 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03-10'!$A$2:$P$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05-10'!$A$2:$P$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06-10'!$A$2:$P$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'07-10'!$A$2:$P$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$E$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -68,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="795">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2657" uniqueCount="903">
   <si>
     <t>NGÀY</t>
   </si>
@@ -2453,6 +2455,330 @@
   </si>
   <si>
     <t>grab</t>
+  </si>
+  <si>
+    <t>Tu Tu</t>
+  </si>
+  <si>
+    <t>HD064689</t>
+  </si>
+  <si>
+    <t>466/39 le van sy f 14</t>
+  </si>
+  <si>
+    <t>07-10-2026</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Thuỳ Trang</t>
+  </si>
+  <si>
+    <t>HD064608</t>
+  </si>
+  <si>
+    <t>41A Huỳnh Tịnh của p19</t>
+  </si>
+  <si>
+    <t>Ngọc Ánh</t>
+  </si>
+  <si>
+    <t>HD064642</t>
+  </si>
+  <si>
+    <t>2/21 phan thúc duyện</t>
+  </si>
+  <si>
+    <t>BN6352</t>
+  </si>
+  <si>
+    <t>HD064708</t>
+  </si>
+  <si>
+    <t>Tú Oanh - fb Không Nói Xâm</t>
+  </si>
+  <si>
+    <t>HD064593</t>
+  </si>
+  <si>
+    <t>69 Dương Đình Nghệ P8</t>
+  </si>
+  <si>
+    <t>AT 07-10</t>
+  </si>
+  <si>
+    <t>Đinh Thị Thu Hà</t>
+  </si>
+  <si>
+    <t>HD064612</t>
+  </si>
+  <si>
+    <t>176/1 Nguyễn Văn Thương, P. Thạnh Mỹ Tây</t>
+  </si>
+  <si>
+    <t>HD064640</t>
+  </si>
+  <si>
+    <t>mỹ huyền</t>
+  </si>
+  <si>
+    <t>HD064774</t>
+  </si>
+  <si>
+    <t>hẻm 2581/27 ấp4 đường huỳnh tấn phát, xã phú xuân</t>
+  </si>
+  <si>
+    <t>Sang - fb Ivy Thụy Pham sale</t>
+  </si>
+  <si>
+    <t>HD064668</t>
+  </si>
+  <si>
+    <t>349/175 Lê Đại Hành Phường Phú Thọ</t>
+  </si>
+  <si>
+    <t>Doan Ngoc Anh Thu</t>
+  </si>
+  <si>
+    <t>HD064813</t>
+  </si>
+  <si>
+    <t>Chung cư homyland2, 307 Nguyễn duy trinh, bình trưng</t>
+  </si>
+  <si>
+    <t>Sea</t>
+  </si>
+  <si>
+    <t>HD064748</t>
+  </si>
+  <si>
+    <t>32/16a đường số 6, P. BHHA</t>
+  </si>
+  <si>
+    <t>Thu Ba DS</t>
+  </si>
+  <si>
+    <t>HD064675</t>
+  </si>
+  <si>
+    <t>395 Bùi Đình Tuý, p14</t>
+  </si>
+  <si>
+    <t>Nhi Nguyễn</t>
+  </si>
+  <si>
+    <t>HD064789</t>
+  </si>
+  <si>
+    <t>128 Hồng Hà, Phường 9</t>
+  </si>
+  <si>
+    <t>chị Thu Dương</t>
+  </si>
+  <si>
+    <t>HD064786</t>
+  </si>
+  <si>
+    <t>158 đào duy anh, P. đức nhuận</t>
+  </si>
+  <si>
+    <t>Linh Dịu Dàng</t>
+  </si>
+  <si>
+    <t>HD064810</t>
+  </si>
+  <si>
+    <t>362/22 lê đức thọ an nhơn</t>
+  </si>
+  <si>
+    <t>Kelly Phan</t>
+  </si>
+  <si>
+    <t>HD064673</t>
+  </si>
+  <si>
+    <t>240/6A lê thánh tôn bến thành</t>
+  </si>
+  <si>
+    <t>Huỳnh Anh</t>
+  </si>
+  <si>
+    <t>HD064778</t>
+  </si>
+  <si>
+    <t>Angelica Lumiere, Vinhome Grand Park, Phường long bình</t>
+  </si>
+  <si>
+    <t>Chip Chip</t>
+  </si>
+  <si>
+    <t>HD064771</t>
+  </si>
+  <si>
+    <t>71/16 thới an 16</t>
+  </si>
+  <si>
+    <t>Trần Thu Hường</t>
+  </si>
+  <si>
+    <t>HD064655</t>
+  </si>
+  <si>
+    <t>124/28 nguyễn văn cừ, p.cầu ông lãnh</t>
+  </si>
+  <si>
+    <t>Vũ Hồng Ly</t>
+  </si>
+  <si>
+    <t>HD064734</t>
+  </si>
+  <si>
+    <t>240/29, Hiệp Thành 13, P Tân Thới Hiệp</t>
+  </si>
+  <si>
+    <t>Cin Vo</t>
+  </si>
+  <si>
+    <t>HD064606</t>
+  </si>
+  <si>
+    <t>268 bà hom p14</t>
+  </si>
+  <si>
+    <t>Bông Bông</t>
+  </si>
+  <si>
+    <t>HD064666</t>
+  </si>
+  <si>
+    <t>Saicon riverside complex (block C1) Số 4 đào trí phú thuận</t>
+  </si>
+  <si>
+    <t>Thu Pham</t>
+  </si>
+  <si>
+    <t>HD064657</t>
+  </si>
+  <si>
+    <t>chung cư Terra Royal 280 nam kỳ khởi nghĩa, phường võ thị sáu</t>
+  </si>
+  <si>
+    <t>HD064688</t>
+  </si>
+  <si>
+    <t>sldraalvinaa_</t>
+  </si>
+  <si>
+    <t>HD064502</t>
+  </si>
+  <si>
+    <t>1 Đường Số 15 Villa 01 David, An Khánh</t>
+  </si>
+  <si>
+    <t>My My</t>
+  </si>
+  <si>
+    <t>HD064651</t>
+  </si>
+  <si>
+    <t>CC TOPAZ ELITE PHOENIX 1A</t>
+  </si>
+  <si>
+    <t>Trang Nguyen</t>
+  </si>
+  <si>
+    <t>HD064597</t>
+  </si>
+  <si>
+    <t>Bệnh viện 1A - lý thường kiệt</t>
+  </si>
+  <si>
+    <t>Ngọc Ngân</t>
+  </si>
+  <si>
+    <t>HD064793</t>
+  </si>
+  <si>
+    <t>87 duong so 79, tan quy</t>
+  </si>
+  <si>
+    <t>Kim Chúc</t>
+  </si>
+  <si>
+    <t>HD064725</t>
+  </si>
+  <si>
+    <t>Hẻm 18B/73 Nguyễn thị minh khai đakao</t>
+  </si>
+  <si>
+    <t>Chi Linh</t>
+  </si>
+  <si>
+    <t>HD064709</t>
+  </si>
+  <si>
+    <t>813 Trần Xuân Soạn</t>
+  </si>
+  <si>
+    <t>Nghi</t>
+  </si>
+  <si>
+    <t>HD064749</t>
+  </si>
+  <si>
+    <t>62 Nguyễn Văn Yến, p Tân Thới Hoà</t>
+  </si>
+  <si>
+    <t>Tranie Phan</t>
+  </si>
+  <si>
+    <t>HD064600</t>
+  </si>
+  <si>
+    <t>1041/19/7 Trần Xuân Soạn</t>
+  </si>
+  <si>
+    <t>Lê Thị Minh Phượng</t>
+  </si>
+  <si>
+    <t>HD064664</t>
+  </si>
+  <si>
+    <t>101/20 đường số 9 phường bình hưng hòa</t>
+  </si>
+  <si>
+    <t>Chau Nguyen</t>
+  </si>
+  <si>
+    <t>HD064811</t>
+  </si>
+  <si>
+    <t>2555 QL1A Phường Tân Hưng Thuận</t>
+  </si>
+  <si>
+    <t>MINZZY</t>
+  </si>
+  <si>
+    <t>XE TOÀN THẮNG VỀ CÀ PHÊ PHONG LONG THÀNH ĐỒNG NAI</t>
+  </si>
+  <si>
+    <t>HOANG ANH</t>
+  </si>
+  <si>
+    <t>385/4 quang trung p go vap</t>
+  </si>
+  <si>
+    <t>vi hồ</t>
+  </si>
+  <si>
+    <t>Nhà xe Minh Quốc</t>
+  </si>
+  <si>
+    <t>at 07-10</t>
+  </si>
+  <si>
+    <t>THU 4</t>
+  </si>
+  <si>
+    <t>NGAY 7-10</t>
   </si>
 </sst>
 </file>
@@ -3039,7 +3365,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="str" cm="1">
-        <f t="array" aca="1" ref="A3:A7" ca="1">_xlfn.LET(
+        <f t="array" aca="1" ref="A3:A8" ca="1">_xlfn.LET(
     _xlpm.start,DATE(B1,--_xlfn.TEXTAFTER(A1," "),1),
     _xlpm.d,_xlfn._xlws.FILTER(
         _xlfn.SEQUENCE(DAY(EOMONTH(_xlpm.start,0)),,_xlpm.start),
@@ -3167,14 +3493,17 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+      <c r="A8" s="3" t="str">
+        <f ca="1"/>
+        <v>07-10</v>
+      </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" s="4" cm="1">
         <f t="array" aca="1" ref="D8" ca="1">IFERROR(SUM(COUNTIF(INDIRECT("'"&amp;A8&amp;"'!M3:M200"),{"*đơn trả*","*hàng tỉnh*"})),0)</f>
@@ -3182,7 +3511,7 @@
       </c>
       <c r="E8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3571,7 +3900,7 @@
       </c>
       <c r="E29" s="5">
         <f ca="1">SUBTOTAL(9,E3:E28)</f>
-        <v>244</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -3588,7 +3917,7 @@
         ),
     0)
 )</f>
-        <v>1083</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -3597,7 +3926,7 @@
       </c>
       <c r="E31" s="5">
         <f ca="1">-E29*2</f>
-        <v>-488</v>
+        <v>-560</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -3606,7 +3935,7 @@
       </c>
       <c r="E32" s="5">
         <f ca="1">SUBTOTAL(9,E30:E31)</f>
-        <v>595</v>
+        <v>669</v>
       </c>
     </row>
   </sheetData>
@@ -17905,4 +18234,2191 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1489BF44-8EF7-4971-A5A2-1BCEF6DB9F6C}">
+  <dimension ref="A1:R65"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="5" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" customWidth="1"/>
+    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B1" s="17" t="s">
+        <v>901</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>902</v>
+      </c>
+      <c r="F1" s="18"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" s="20"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="20"/>
+      <c r="B3" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>807</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>808</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>809</v>
+      </c>
+      <c r="F3" s="21">
+        <v>11</v>
+      </c>
+      <c r="G3" s="21">
+        <v>0</v>
+      </c>
+      <c r="H3" s="21">
+        <v>25</v>
+      </c>
+      <c r="I3" s="21">
+        <f t="shared" ref="I3:I39" si="0">G3-H3</f>
+        <v>-25</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20">
+        <v>1</v>
+      </c>
+      <c r="R3" s="8">
+        <f>H3</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>815</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>816</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>817</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="G4" s="21">
+        <v>825</v>
+      </c>
+      <c r="H4" s="21">
+        <v>35</v>
+      </c>
+      <c r="I4" s="21">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K4" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="20"/>
+      <c r="B5" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>818</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>819</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>820</v>
+      </c>
+      <c r="F5" s="21">
+        <v>11</v>
+      </c>
+      <c r="G5" s="21">
+        <v>3780</v>
+      </c>
+      <c r="H5" s="21">
+        <v>35</v>
+      </c>
+      <c r="I5" s="21">
+        <f t="shared" si="0"/>
+        <v>3745</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L5" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M5" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20">
+        <v>1</v>
+      </c>
+      <c r="R5" s="8">
+        <f>H5</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="20"/>
+      <c r="B6" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>824</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>825</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>826</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="21">
+        <v>0</v>
+      </c>
+      <c r="H6" s="21">
+        <v>30</v>
+      </c>
+      <c r="I6" s="21">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J6" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L6" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20">
+        <v>1</v>
+      </c>
+      <c r="R6" s="8">
+        <f>H6</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>851</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>852</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>853</v>
+      </c>
+      <c r="F7" s="21">
+        <v>12</v>
+      </c>
+      <c r="G7" s="21">
+        <v>1380</v>
+      </c>
+      <c r="H7" s="21">
+        <v>30</v>
+      </c>
+      <c r="I7" s="21">
+        <f t="shared" si="0"/>
+        <v>1350</v>
+      </c>
+      <c r="J7" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L7" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>854</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>855</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>856</v>
+      </c>
+      <c r="F8" s="21">
+        <v>6</v>
+      </c>
+      <c r="G8" s="21">
+        <v>865</v>
+      </c>
+      <c r="H8" s="21">
+        <v>25</v>
+      </c>
+      <c r="I8" s="21">
+        <f t="shared" si="0"/>
+        <v>840</v>
+      </c>
+      <c r="J8" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L8" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>857</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>858</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>859</v>
+      </c>
+      <c r="F9" s="21">
+        <v>7</v>
+      </c>
+      <c r="G9" s="21">
+        <v>910</v>
+      </c>
+      <c r="H9" s="21">
+        <v>30</v>
+      </c>
+      <c r="I9" s="21">
+        <f t="shared" si="0"/>
+        <v>880</v>
+      </c>
+      <c r="J9" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L9" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>873</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>874</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>875</v>
+      </c>
+      <c r="F10" s="21">
+        <v>7</v>
+      </c>
+      <c r="G10" s="21">
+        <v>850</v>
+      </c>
+      <c r="H10" s="21">
+        <v>30</v>
+      </c>
+      <c r="I10" s="21">
+        <f t="shared" si="0"/>
+        <v>820</v>
+      </c>
+      <c r="J10" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K10" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L10" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>882</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>883</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>884</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="G11" s="21">
+        <v>915</v>
+      </c>
+      <c r="H11" s="21">
+        <v>25</v>
+      </c>
+      <c r="I11" s="21">
+        <f t="shared" si="0"/>
+        <v>890</v>
+      </c>
+      <c r="J11" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L11" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>888</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>889</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>890</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="21">
+        <v>1410</v>
+      </c>
+      <c r="H12" s="21">
+        <v>30</v>
+      </c>
+      <c r="I12" s="21">
+        <f t="shared" si="0"/>
+        <v>1380</v>
+      </c>
+      <c r="J12" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K12" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L12" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M12" s="20"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>891</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>892</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>893</v>
+      </c>
+      <c r="F13" s="21">
+        <v>12</v>
+      </c>
+      <c r="G13" s="21">
+        <v>490</v>
+      </c>
+      <c r="H13" s="21">
+        <v>30</v>
+      </c>
+      <c r="I13" s="21">
+        <f t="shared" si="0"/>
+        <v>460</v>
+      </c>
+      <c r="J13" s="20" t="s">
+        <v>810</v>
+      </c>
+      <c r="K13" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L13" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M13" s="20"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="20"/>
+      <c r="P13" s="20"/>
+      <c r="Q13" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>799</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>800</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>801</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="21">
+        <v>1340</v>
+      </c>
+      <c r="H14" s="21">
+        <v>20</v>
+      </c>
+      <c r="I14" s="21">
+        <f t="shared" si="0"/>
+        <v>1320</v>
+      </c>
+      <c r="J14" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L14" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M14" s="20"/>
+      <c r="N14" s="20"/>
+      <c r="O14" s="20"/>
+      <c r="P14" s="20"/>
+      <c r="Q14" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="20"/>
+      <c r="B15" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>805</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>806</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="21">
+        <v>12</v>
+      </c>
+      <c r="G15" s="21">
+        <v>0</v>
+      </c>
+      <c r="H15" s="21">
+        <v>30</v>
+      </c>
+      <c r="I15" s="21">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J15" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L15" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="20"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="20">
+        <v>1</v>
+      </c>
+      <c r="R15" s="8">
+        <f>H15</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>811</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>812</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>813</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="21">
+        <v>1010</v>
+      </c>
+      <c r="H16" s="21">
+        <v>20</v>
+      </c>
+      <c r="I16" s="21">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L16" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M16" s="20"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="20"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="20"/>
+      <c r="B17" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>821</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>822</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>823</v>
+      </c>
+      <c r="F17" s="21">
+        <v>2</v>
+      </c>
+      <c r="G17" s="21">
+        <v>820</v>
+      </c>
+      <c r="H17" s="21">
+        <v>30</v>
+      </c>
+      <c r="I17" s="21">
+        <f t="shared" si="0"/>
+        <v>790</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L17" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="20"/>
+      <c r="Q17" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>827</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>828</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>829</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="21">
+        <v>0</v>
+      </c>
+      <c r="H18" s="21">
+        <v>20</v>
+      </c>
+      <c r="I18" s="21">
+        <f t="shared" si="0"/>
+        <v>-20</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L18" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M18" s="20"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="20"/>
+      <c r="P18" s="20"/>
+      <c r="Q18" s="20">
+        <v>1</v>
+      </c>
+      <c r="R18" s="8">
+        <f>H18</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>836</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>837</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>838</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="G19" s="21">
+        <v>1485</v>
+      </c>
+      <c r="H19" s="21">
+        <v>25</v>
+      </c>
+      <c r="I19" s="21">
+        <f t="shared" si="0"/>
+        <v>1460</v>
+      </c>
+      <c r="J19" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K19" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="20"/>
+      <c r="Q19" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="20"/>
+      <c r="B20" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>842</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>843</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>844</v>
+      </c>
+      <c r="F20" s="21">
+        <v>9</v>
+      </c>
+      <c r="G20" s="21">
+        <v>0</v>
+      </c>
+      <c r="H20" s="21">
+        <v>30</v>
+      </c>
+      <c r="I20" s="21">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J20" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L20" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M20" s="20"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="20"/>
+      <c r="P20" s="20"/>
+      <c r="Q20" s="20">
+        <v>1</v>
+      </c>
+      <c r="R20" s="8">
+        <f>H20</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>845</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>846</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>847</v>
+      </c>
+      <c r="F21" s="21">
+        <v>12</v>
+      </c>
+      <c r="G21" s="21">
+        <v>1710</v>
+      </c>
+      <c r="H21" s="21">
+        <v>30</v>
+      </c>
+      <c r="I21" s="21">
+        <f t="shared" si="0"/>
+        <v>1680</v>
+      </c>
+      <c r="J21" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K21" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L21" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M21" s="20"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="20"/>
+      <c r="P21" s="20"/>
+      <c r="Q21" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>864</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>865</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>866</v>
+      </c>
+      <c r="F22" s="21">
+        <v>2</v>
+      </c>
+      <c r="G22" s="21">
+        <v>0</v>
+      </c>
+      <c r="H22" s="21">
+        <v>30</v>
+      </c>
+      <c r="I22" s="21">
+        <f t="shared" si="0"/>
+        <v>-30</v>
+      </c>
+      <c r="J22" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K22" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M22" s="20"/>
+      <c r="N22" s="20"/>
+      <c r="O22" s="20"/>
+      <c r="P22" s="20"/>
+      <c r="Q22" s="20">
+        <v>1</v>
+      </c>
+      <c r="R22" s="8">
+        <f t="shared" ref="R22:R23" si="1">H22</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>894</v>
+      </c>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20" t="s">
+        <v>895</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G23" s="21">
+        <v>0</v>
+      </c>
+      <c r="H23" s="21">
+        <v>25</v>
+      </c>
+      <c r="I23" s="21">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J23" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K23" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L23" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20"/>
+      <c r="P23" s="20"/>
+      <c r="Q23" s="20">
+        <v>1</v>
+      </c>
+      <c r="R23" s="8">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>896</v>
+      </c>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20" t="s">
+        <v>897</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="G24" s="21">
+        <v>30</v>
+      </c>
+      <c r="H24" s="21">
+        <v>30</v>
+      </c>
+      <c r="I24" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K24" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L24" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="20"/>
+      <c r="P24" s="20"/>
+      <c r="Q24" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>898</v>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20" t="s">
+        <v>899</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="G25" s="21">
+        <v>0</v>
+      </c>
+      <c r="H25" s="21">
+        <v>40</v>
+      </c>
+      <c r="I25" s="21">
+        <f t="shared" si="0"/>
+        <v>-40</v>
+      </c>
+      <c r="J25" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="K25" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L25" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M25" s="20"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="20"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20">
+        <v>1</v>
+      </c>
+      <c r="R25" s="8">
+        <f>H25</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>795</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>796</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>797</v>
+      </c>
+      <c r="F26" s="21">
+        <v>3</v>
+      </c>
+      <c r="G26" s="21">
+        <v>1765</v>
+      </c>
+      <c r="H26" s="21">
+        <v>25</v>
+      </c>
+      <c r="I26" s="21">
+        <f t="shared" si="0"/>
+        <v>1740</v>
+      </c>
+      <c r="J26" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K26" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L26" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M26" s="20"/>
+      <c r="N26" s="20"/>
+      <c r="O26" s="20"/>
+      <c r="P26" s="20"/>
+      <c r="Q26" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>802</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>803</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>804</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="G27" s="21">
+        <v>365</v>
+      </c>
+      <c r="H27" s="21">
+        <v>25</v>
+      </c>
+      <c r="I27" s="21">
+        <f t="shared" si="0"/>
+        <v>340</v>
+      </c>
+      <c r="J27" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K27" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L27" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M27" s="23" t="s">
+        <v>374</v>
+      </c>
+      <c r="N27" s="20"/>
+      <c r="O27" s="20"/>
+      <c r="P27" s="20"/>
+      <c r="Q27" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>802</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>814</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>804</v>
+      </c>
+      <c r="F28" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="G28" s="21">
+        <v>0</v>
+      </c>
+      <c r="H28" s="21">
+        <v>0</v>
+      </c>
+      <c r="I28" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K28" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L28" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M28" s="23" t="s">
+        <v>374</v>
+      </c>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
+      <c r="P28" s="20"/>
+      <c r="Q28" s="20">
+        <v>1</v>
+      </c>
+      <c r="R28" s="8">
+        <f>H28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" s="20"/>
+      <c r="B29" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>830</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>831</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>832</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="G29" s="21">
+        <v>480</v>
+      </c>
+      <c r="H29" s="21">
+        <v>20</v>
+      </c>
+      <c r="I29" s="21">
+        <f t="shared" si="0"/>
+        <v>460</v>
+      </c>
+      <c r="J29" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K29" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L29" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M29" s="20"/>
+      <c r="N29" s="20"/>
+      <c r="O29" s="20"/>
+      <c r="P29" s="20"/>
+      <c r="Q29" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" s="20"/>
+      <c r="B30" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>833</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>834</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>835</v>
+      </c>
+      <c r="F30" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="G30" s="21">
+        <v>4520</v>
+      </c>
+      <c r="H30" s="21">
+        <v>35</v>
+      </c>
+      <c r="I30" s="21">
+        <f t="shared" si="0"/>
+        <v>4485</v>
+      </c>
+      <c r="J30" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K30" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L30" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M30" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="N30" s="20"/>
+      <c r="O30" s="20"/>
+      <c r="P30" s="20"/>
+      <c r="Q30" s="20">
+        <v>1</v>
+      </c>
+      <c r="R30" s="8">
+        <f>H30</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31" s="20"/>
+      <c r="B31" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>839</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>840</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>841</v>
+      </c>
+      <c r="F31" s="21">
+        <v>1</v>
+      </c>
+      <c r="G31" s="21">
+        <v>0</v>
+      </c>
+      <c r="H31" s="21">
+        <v>25</v>
+      </c>
+      <c r="I31" s="21">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J31" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K31" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L31" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M31" s="20"/>
+      <c r="N31" s="20"/>
+      <c r="O31" s="20"/>
+      <c r="P31" s="20"/>
+      <c r="Q31" s="20">
+        <v>1</v>
+      </c>
+      <c r="R31" s="8">
+        <f>H31</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" s="20"/>
+      <c r="B32" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>848</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>849</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>850</v>
+      </c>
+      <c r="F32" s="21">
+        <v>1</v>
+      </c>
+      <c r="G32" s="21">
+        <v>1015</v>
+      </c>
+      <c r="H32" s="21">
+        <v>25</v>
+      </c>
+      <c r="I32" s="21">
+        <f t="shared" si="0"/>
+        <v>990</v>
+      </c>
+      <c r="J32" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K32" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L32" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M32" s="20"/>
+      <c r="N32" s="20"/>
+      <c r="O32" s="20"/>
+      <c r="P32" s="20"/>
+      <c r="Q32" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" s="20"/>
+      <c r="B33" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>860</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>861</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>862</v>
+      </c>
+      <c r="F33" s="21">
+        <v>3</v>
+      </c>
+      <c r="G33" s="21">
+        <v>1315</v>
+      </c>
+      <c r="H33" s="21">
+        <v>25</v>
+      </c>
+      <c r="I33" s="21">
+        <f t="shared" si="0"/>
+        <v>1290</v>
+      </c>
+      <c r="J33" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K33" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L33" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M33" s="20"/>
+      <c r="N33" s="20"/>
+      <c r="O33" s="20"/>
+      <c r="P33" s="20"/>
+      <c r="Q33" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="24"/>
+      <c r="B34" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>710</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>863</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>712</v>
+      </c>
+      <c r="F34" s="25">
+        <v>3</v>
+      </c>
+      <c r="G34" s="25">
+        <v>0</v>
+      </c>
+      <c r="H34" s="25">
+        <v>25</v>
+      </c>
+      <c r="I34" s="25">
+        <f t="shared" si="0"/>
+        <v>-25</v>
+      </c>
+      <c r="J34" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="K34" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="L34" s="24" t="s">
+        <v>798</v>
+      </c>
+      <c r="M34" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="N34" s="24"/>
+      <c r="O34" s="24"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24">
+        <v>1</v>
+      </c>
+      <c r="R34" s="34">
+        <f>H34</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="20"/>
+      <c r="B35" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="20" t="s">
+        <v>867</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>868</v>
+      </c>
+      <c r="E35" s="20" t="s">
+        <v>869</v>
+      </c>
+      <c r="F35" s="21">
+        <v>7</v>
+      </c>
+      <c r="G35" s="21">
+        <v>890</v>
+      </c>
+      <c r="H35" s="21">
+        <v>30</v>
+      </c>
+      <c r="I35" s="21">
+        <f t="shared" si="0"/>
+        <v>860</v>
+      </c>
+      <c r="J35" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K35" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L35" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M35" s="20"/>
+      <c r="N35" s="20"/>
+      <c r="O35" s="20"/>
+      <c r="P35" s="20"/>
+      <c r="Q35" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" s="20"/>
+      <c r="B36" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>870</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>871</v>
+      </c>
+      <c r="E36" s="20" t="s">
+        <v>872</v>
+      </c>
+      <c r="F36" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="G36" s="21">
+        <v>515</v>
+      </c>
+      <c r="H36" s="21">
+        <v>25</v>
+      </c>
+      <c r="I36" s="21">
+        <f t="shared" si="0"/>
+        <v>490</v>
+      </c>
+      <c r="J36" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K36" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L36" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M36" s="20"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="20"/>
+      <c r="Q36" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37" s="20"/>
+      <c r="B37" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>876</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>877</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>878</v>
+      </c>
+      <c r="F37" s="21">
+        <v>1</v>
+      </c>
+      <c r="G37" s="21">
+        <v>905</v>
+      </c>
+      <c r="H37" s="21">
+        <v>25</v>
+      </c>
+      <c r="I37" s="21">
+        <f t="shared" si="0"/>
+        <v>880</v>
+      </c>
+      <c r="J37" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K37" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L37" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M37" s="20"/>
+      <c r="N37" s="20"/>
+      <c r="O37" s="20"/>
+      <c r="P37" s="20"/>
+      <c r="Q37" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="24"/>
+      <c r="B38" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>879</v>
+      </c>
+      <c r="D38" s="24" t="s">
+        <v>880</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>881</v>
+      </c>
+      <c r="F38" s="25">
+        <v>7</v>
+      </c>
+      <c r="G38" s="25">
+        <v>30</v>
+      </c>
+      <c r="H38" s="25">
+        <v>30</v>
+      </c>
+      <c r="I38" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J38" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="K38" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="L38" s="24" t="s">
+        <v>798</v>
+      </c>
+      <c r="M38" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="N38" s="24"/>
+      <c r="O38" s="24"/>
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" s="20"/>
+      <c r="B39" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>885</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>886</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>887</v>
+      </c>
+      <c r="F39" s="21">
+        <v>7</v>
+      </c>
+      <c r="G39" s="21">
+        <v>760</v>
+      </c>
+      <c r="H39" s="21">
+        <v>30</v>
+      </c>
+      <c r="I39" s="21">
+        <f t="shared" si="0"/>
+        <v>730</v>
+      </c>
+      <c r="J39" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="K39" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="L39" s="20" t="s">
+        <v>798</v>
+      </c>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
+      <c r="O39" s="20"/>
+      <c r="P39" s="20"/>
+      <c r="Q39" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D41" s="9">
+        <f>COUNTA(D3:D39)</f>
+        <v>34</v>
+      </c>
+      <c r="G41" s="9">
+        <f t="shared" ref="G41:Q41" si="2">SUBTOTAL(9,G3:G39)</f>
+        <v>30380</v>
+      </c>
+      <c r="H41" s="9">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
+      <c r="I41" s="9">
+        <f t="shared" si="2"/>
+        <v>29380</v>
+      </c>
+      <c r="J41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P41" s="9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q41" s="9">
+        <f t="shared" si="2"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H42">
+        <f>-6*17</f>
+        <v>-102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C43" s="45" t="s">
+        <v>189</v>
+      </c>
+      <c r="D43" s="45"/>
+      <c r="E43" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="H43">
+        <f>-4*25</f>
+        <v>-100</v>
+      </c>
+      <c r="K43" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="L43" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M43" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="O43" s="10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>798</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="C44" s="46">
+        <f>SUMIFS(I$3:I$39,B$3:B$39,A$43,L$3:L$39,A$44)</f>
+        <v>29380</v>
+      </c>
+      <c r="D44" s="46"/>
+      <c r="E44" s="12">
+        <f>SUMIFS(Q$3:Q$39,B$3:B$39,A$43,L$3:L$39,A$44)</f>
+        <v>37</v>
+      </c>
+      <c r="F44" t="s">
+        <v>194</v>
+      </c>
+      <c r="H44">
+        <f>-1*30</f>
+        <v>-30</v>
+      </c>
+      <c r="K44" t="s">
+        <v>195</v>
+      </c>
+      <c r="L44">
+        <f>SUMIFS(G$3:G$39,J$3:J$39,K$43)</f>
+        <v>12560</v>
+      </c>
+      <c r="M44">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$43)-INT(COUNTIFS(J$3:J$39,K$43,M$3:M$39,"*gộp*")/2)</f>
+        <v>13</v>
+      </c>
+      <c r="O44" t="s">
+        <v>30</v>
+      </c>
+      <c r="P44">
+        <f>L49</f>
+        <v>12280</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B45" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C45" s="47">
+        <v>0</v>
+      </c>
+      <c r="D45" s="47"/>
+      <c r="K45" t="s">
+        <v>197</v>
+      </c>
+      <c r="L45">
+        <f>-SUMIFS(H$3:H$39,J$3:J$39,K$43)+M45*5</f>
+        <v>-280</v>
+      </c>
+      <c r="M45">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$43)-INT(COUNTIFS(J$3:J$39,K$43,M$3:M$39,"*gộp*")/2)</f>
+        <v>13</v>
+      </c>
+      <c r="O45" t="s">
+        <v>31</v>
+      </c>
+      <c r="P45">
+        <f>L57</f>
+        <v>6053</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B46" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C46" s="47">
+        <f>-SUMIFS(I$3:I$39,B$3:B$39,A$43,P$3:P$39,"xx",N$3:N$39,"x")</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="47"/>
+      <c r="E46" s="13">
+        <f>SUMIFS(Q$3:Q$39,B$3:B$39,A$43,P$3:P$39,"xx",N$3:N$39,"x")</f>
+        <v>0</v>
+      </c>
+      <c r="K46" t="s">
+        <v>200</v>
+      </c>
+      <c r="L46">
+        <f>-M46*2</f>
+        <v>0</v>
+      </c>
+      <c r="M46">
+        <f>COUNTIFS(K$3:K$39,K$43,L$3:L$39,A$44)-(COUNTIFS(K$3:K$39,K$43,M$3:M$39,"*gộp*")/2)-COUNTIFS(K$3:K$39,K$43,M$3:M$39,"*đơn trả*")-COUNTIFS(K$3:K$39,K$43,M$3:M$39,"*hàng tỉnh*")</f>
+        <v>0</v>
+      </c>
+      <c r="O46" t="s">
+        <v>900</v>
+      </c>
+      <c r="P46">
+        <f>L65</f>
+        <v>11193</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B47" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C47" s="45">
+        <f>SUBTOTAL(9,C44:C46)</f>
+        <v>29380</v>
+      </c>
+      <c r="D47" s="45"/>
+      <c r="E47">
+        <f>E44</f>
+        <v>37</v>
+      </c>
+      <c r="K47" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="O47" t="s">
+        <v>203</v>
+      </c>
+      <c r="P47">
+        <f>-C51</f>
+        <v>-29380</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B48" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C48" s="43"/>
+      <c r="D48" s="43"/>
+      <c r="K48" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="O48" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="P48" s="10">
+        <f>SUBTOTAL(9,P44:P47)</f>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B49" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C49" s="43"/>
+      <c r="D49" s="43"/>
+      <c r="L49" s="16">
+        <f>SUBTOTAL(9,L44:L48)</f>
+        <v>12280</v>
+      </c>
+      <c r="M49" s="16">
+        <f>M44</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B51" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="C51" s="44">
+        <f>C47+C48+C49</f>
+        <v>29380</v>
+      </c>
+      <c r="D51" s="44"/>
+      <c r="E51" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="K51" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L51" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M51" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K52" t="s">
+        <v>195</v>
+      </c>
+      <c r="L52">
+        <f>SUMIFS(G$3:G$39,J$3:J$39,K$51)</f>
+        <v>6395</v>
+      </c>
+      <c r="M52">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$51)-INT(COUNTIFS(J$3:J$39,K$51,M$3:M$39,"*gộp*")/2)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K53" t="s">
+        <v>197</v>
+      </c>
+      <c r="L53">
+        <f>-SUMIFS(H$3:H$39,J$3:J$39,K$51)+M53*5</f>
+        <v>-270</v>
+      </c>
+      <c r="M53">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$51)-INT(COUNTIFS(J$3:J$39,K$51,M$3:M$39,"*gộp*")/2)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K54" t="s">
+        <v>200</v>
+      </c>
+      <c r="L54">
+        <f>-M54*2</f>
+        <v>-72</v>
+      </c>
+      <c r="M54">
+        <f>COUNTIFS(K$3:K$39,K$51,L$3:L$39,A$44)-(COUNTIFS(K$3:K$39,K$51,M$3:M$39,"*gộp*")/2)-COUNTIFS(K$3:K$39,K$51,M$3:M$39,"*đơn trả*")-COUNTIFS(K$3:K$39,K$51,M$3:M$39,"*hàng tỉnh*")</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K55" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K56" s="13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="L57" s="16">
+        <f>SUBTOTAL(9,L52:L56)</f>
+        <v>6053</v>
+      </c>
+      <c r="M57" s="16">
+        <f>M52</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K59" s="11" t="s">
+        <v>810</v>
+      </c>
+      <c r="L59" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M59" s="11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K60" t="s">
+        <v>195</v>
+      </c>
+      <c r="L60">
+        <f>SUMIFS(G$3:G$39,J$3:J$39,K$59)</f>
+        <v>11425</v>
+      </c>
+      <c r="M60">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$59)-INT(COUNTIFS(J$3:J$39,K$59,M$3:M$39,"*gộp*")/2)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K61" t="s">
+        <v>197</v>
+      </c>
+      <c r="L61">
+        <f>SUM(H42:H44)</f>
+        <v>-232</v>
+      </c>
+      <c r="M61">
+        <f>SUMIFS(Q$3:Q$39,J$3:J$39,K$59)-INT(COUNTIFS(J$3:J$39,K$59,M$3:M$39,"*gộp*")/2)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K62" t="s">
+        <v>200</v>
+      </c>
+      <c r="L62">
+        <f>-M62*2</f>
+        <v>0</v>
+      </c>
+      <c r="M62">
+        <f>COUNTIFS(K$3:K$39,K$59,L$3:L$39,A$44)-(COUNTIFS(K$3:K$39,K$59,M$3:M$39,"*gộp*")/2)-COUNTIFS(K$3:K$39,K$59,M$3:M$39,"*đơn trả*")-COUNTIFS(K$3:K$39,K$59,M$3:M$39,"*hàng tỉnh*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K63" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K64" s="13" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="65" spans="12:13" x14ac:dyDescent="0.25">
+      <c r="L65" s="16">
+        <f>SUBTOTAL(9,L60:L64)</f>
+        <v>11193</v>
+      </c>
+      <c r="M65" s="16">
+        <f>M60</f>
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:P39" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:P39">
+      <sortCondition ref="J2:J39"/>
+    </sortState>
+  </autoFilter>
+  <mergeCells count="8">
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+</worksheet>
 </file>
</xml_diff>